<commit_message>
Fix date mismatch on Sept 10 doc-collection sub-activities
Four sub-activities noted as "Due Thu Sept 10 EOD" were dated to their
parent activity's full week instead of the actual Sept 8-10 window
that note refers to. Also moved the DataVisor doc-collection
sub-activity to Week 1 (when the request goes out) rather than Week 3
(when the parent design activity starts on the gantt).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Msiz5p6hoKmmUHZyLJTkqb
</commit_message>
<xml_diff>
--- a/Beem Visa Debit - Transformation Phase Project Plan.xlsx
+++ b/Beem Visa Debit - Transformation Phase Project Plan.xlsx
@@ -724,7 +724,7 @@
         <v>46273</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>46279</v>
+        <v>46275</v>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
@@ -902,10 +902,10 @@
         </is>
       </c>
       <c r="F11" s="9" t="n">
-        <v>46286</v>
+        <v>46273</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>46292</v>
+        <v>46275</v>
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
@@ -1707,7 +1707,7 @@
         <v>46273</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>46279</v>
+        <v>46275</v>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
@@ -2332,7 +2332,7 @@
         <v>46273</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>46279</v>
+        <v>46275</v>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>

</xml_diff>